<commit_message>
somewhat done, but not perfect
</commit_message>
<xml_diff>
--- a/mha.xlsx
+++ b/mha.xlsx
@@ -595,7 +595,7 @@
         <v>3.3802550348452</v>
       </c>
       <c r="N2" t="n">
-        <v>39.3</v>
+        <v>43.56</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
@@ -606,13 +606,13 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="n">
-        <v>201</v>
+        <v>223.4</v>
       </c>
       <c r="X2" t="n">
-        <v>2.578891832311018</v>
+        <v>2.09</v>
       </c>
       <c r="Y2" t="n">
-        <v>10.70040506679986</v>
+        <v>6.44</v>
       </c>
     </row>
     <row r="3">
@@ -660,7 +660,7 @@
         <v>0.482582704350119</v>
       </c>
       <c r="N3" t="n">
-        <v>36.6</v>
+        <v>37.77</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
@@ -671,13 +671,13 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="n">
-        <v>178.6</v>
+        <v>201</v>
       </c>
       <c r="X3" t="n">
-        <v>2.965986451718299</v>
+        <v>2.34</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.696781390588743</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="4">
@@ -713,7 +713,7 @@
         <v>-1</v>
       </c>
       <c r="J4" t="n">
-        <v>36.6</v>
+        <v>37.77</v>
       </c>
       <c r="K4" t="n">
         <v>223.4</v>
@@ -725,7 +725,7 @@
         <v>3.77520674788275</v>
       </c>
       <c r="N4" t="n">
-        <v>15.41</v>
+        <v>29.87</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
@@ -736,13 +736,13 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="n">
-        <v>160.8</v>
+        <v>201</v>
       </c>
       <c r="X4" t="n">
-        <v>2.981998380250725</v>
+        <v>1.91</v>
       </c>
       <c r="Y4" t="n">
-        <v>20.19238387517242</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="5">
@@ -778,7 +778,7 @@
         <v>-1</v>
       </c>
       <c r="J5" t="n">
-        <v>15.41</v>
+        <v>43.56</v>
       </c>
       <c r="K5" t="n">
         <v>201</v>
@@ -790,7 +790,7 @@
         <v>2.58242274762665</v>
       </c>
       <c r="N5" t="n">
-        <v>-13.49</v>
+        <v>37.55</v>
       </c>
       <c r="O5" t="n">
         <v>32</v>
@@ -815,13 +815,13 @@
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>125</v>
+        <v>178.6</v>
       </c>
       <c r="X5" t="n">
-        <v>2.69851719745223</v>
+        <v>1.32</v>
       </c>
       <c r="Y5" t="n">
-        <v>27.90332113708621</v>
+        <v>5.01</v>
       </c>
     </row>
     <row r="6">
@@ -857,7 +857,7 @@
         <v>-1</v>
       </c>
       <c r="J6" t="n">
-        <v>-13.49</v>
+        <v>34.25</v>
       </c>
       <c r="K6" t="n">
         <v>160.8</v>
@@ -869,7 +869,7 @@
         <v>0.774921997561535</v>
       </c>
       <c r="N6" t="n">
-        <v>-24.28</v>
+        <v>32.53</v>
       </c>
       <c r="O6" t="n">
         <v>49</v>
@@ -896,13 +896,13 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>96.8</v>
+        <v>160.8</v>
       </c>
       <c r="X6" t="n">
-        <v>2.468990319045591</v>
+        <v>0.52</v>
       </c>
       <c r="Y6" t="n">
-        <v>9.790978106118269</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="7">
@@ -938,7 +938,7 @@
         <v>-1</v>
       </c>
       <c r="J7" t="n">
-        <v>-24.28</v>
+        <v>31.98</v>
       </c>
       <c r="K7" t="n">
         <v>96.8</v>
@@ -950,7 +950,7 @@
         <v>7.46654022259542</v>
       </c>
       <c r="N7" t="n">
-        <v>-33.5</v>
+        <v>30.71</v>
       </c>
       <c r="O7" t="n">
         <v>49</v>
@@ -977,13 +977,13 @@
         <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>96.8</v>
+        <v>160.8</v>
       </c>
       <c r="X7" t="n">
-        <v>1.443246584823963</v>
+        <v>0.37</v>
       </c>
       <c r="Y7" t="n">
-        <v>8.213194244854957</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="8">
@@ -1019,7 +1019,7 @@
         <v>-1</v>
       </c>
       <c r="J8" t="n">
-        <v>-33.5</v>
+        <v>29.71</v>
       </c>
       <c r="K8" t="n">
         <v>96.8</v>
@@ -1031,7 +1031,7 @@
         <v>2.83233969772578</v>
       </c>
       <c r="N8" t="n">
-        <v>-37.61</v>
+        <v>28.44</v>
       </c>
       <c r="O8" t="n">
         <v>46</v>
@@ -1058,13 +1058,13 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>96.8</v>
+        <v>160.8</v>
       </c>
       <c r="X8" t="n">
-        <v>1.025743734221628</v>
+        <v>0.37</v>
       </c>
       <c r="Y8" t="n">
-        <v>3.115573667498354</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="9">
@@ -1100,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>-37.61</v>
+        <v>32.53</v>
       </c>
       <c r="K9" t="n">
         <v>96.8</v>
@@ -1112,7 +1112,7 @@
         <v>4.16428009425356</v>
       </c>
       <c r="N9" t="n">
-        <v>-42.19</v>
+        <v>30.24</v>
       </c>
       <c r="O9" t="n">
         <v>50</v>
@@ -1139,13 +1139,13 @@
         <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>96.8</v>
+        <v>160.8</v>
       </c>
       <c r="X9" t="n">
-        <v>1.022480931090903</v>
+        <v>0.37</v>
       </c>
       <c r="Y9" t="n">
-        <v>4.580708103678916</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="10">
@@ -1181,7 +1181,7 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>-42.19</v>
+        <v>30.22</v>
       </c>
       <c r="K10" t="n">
         <v>96.8</v>
@@ -1193,7 +1193,7 @@
         <v>0.988234001066137</v>
       </c>
       <c r="N10" t="n">
-        <v>-42.28</v>
+        <v>30.67</v>
       </c>
       <c r="O10" t="n">
         <v>68</v>
@@ -1220,13 +1220,13 @@
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>96.8</v>
+        <v>111.6</v>
       </c>
       <c r="X10" t="n">
-        <v>1.021801180438669</v>
+        <v>0.77</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.087057401172751</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="11">
@@ -1262,7 +1262,7 @@
         <v>-2</v>
       </c>
       <c r="J11" t="n">
-        <v>-42.28</v>
+        <v>37.55</v>
       </c>
       <c r="K11" t="n">
         <v>96.8</v>
@@ -1274,7 +1274,7 @@
         <v>3.04579901156206</v>
       </c>
       <c r="N11" t="n">
-        <v>-47.63</v>
+        <v>33.86</v>
       </c>
       <c r="O11" t="n">
         <v>68</v>
@@ -1301,13 +1301,13 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>96.8</v>
+        <v>111.6</v>
       </c>
       <c r="X11" t="n">
-        <v>1.008885918046216</v>
+        <v>0.76</v>
       </c>
       <c r="Y11" t="n">
-        <v>3.350378912718262</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="12">
@@ -1343,7 +1343,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>-47.63</v>
+        <v>32.2</v>
       </c>
       <c r="K12" t="n">
         <v>96.8</v>
@@ -1355,7 +1355,7 @@
         <v>0.120562661968526</v>
       </c>
       <c r="N12" t="n">
-        <v>-47.76</v>
+        <v>32.07</v>
       </c>
       <c r="O12" t="n">
         <v>66</v>
@@ -1385,10 +1385,10 @@
         <v>96.8</v>
       </c>
       <c r="X12" t="n">
-        <v>0.898902262514699</v>
+        <v>0.9</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.132618928165379</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="13">
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>-47.76</v>
+        <v>33.86</v>
       </c>
       <c r="K13" t="n">
         <v>96.8</v>
@@ -1436,7 +1436,7 @@
         <v>4.60872735473449</v>
       </c>
       <c r="N13" t="n">
-        <v>-52.83</v>
+        <v>28.79</v>
       </c>
       <c r="O13" t="n">
         <v>65</v>
@@ -1466,10 +1466,10 @@
         <v>96.8</v>
       </c>
       <c r="X13" t="n">
-        <v>0.9691884799557303</v>
+        <v>0.97</v>
       </c>
       <c r="Y13" t="n">
-        <v>5.069600090207937</v>
+        <v>5.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>